<commit_message>
changes but not working
</commit_message>
<xml_diff>
--- a/UCAS mentee form.xlsx
+++ b/UCAS mentee form.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imperiallondon-my.sharepoint.com/personal/hm1425_ic_ac_uk/Documents/STEMM/Term 1/UCAS mentoring testing/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imperiallondon-my.sharepoint.com/personal/hm1425_ic_ac_uk/Documents/STEMM/Term 1/UCAS mentoring testing/Matching Algorithm/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{AD74628D-BE06-4FC1-BE04-2187DD70E9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13AFE710-26B6-44C8-8F84-35032937E573}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD74628D-BE06-4FC1-BE04-2187DD70E9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="24192" yWindow="2880" windowWidth="21600" windowHeight="11832" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="33">
   <si>
     <t>ID</t>
   </si>
@@ -45,94 +45,85 @@
     <t>Last modified time</t>
   </si>
   <si>
-    <t>Faculty </t>
-  </si>
-  <si>
-    <t>Engineerings</t>
-  </si>
-  <si>
-    <t>Medicines</t>
-  </si>
-  <si>
-    <t>NatSci</t>
-  </si>
-  <si>
-    <t>Business </t>
-  </si>
-  <si>
-    <t>Okay with someone in Faculty but not desired course? </t>
+    <t>Name2</t>
+  </si>
+  <si>
+    <t>Email2</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>Course applying for</t>
   </si>
   <si>
     <t>anonymous</t>
   </si>
   <si>
-    <t>jj1</t>
-  </si>
-  <si>
-    <t>Engineering</t>
-  </si>
-  <si>
-    <t>mecheng </t>
-  </si>
-  <si>
-    <t>Yes</t>
+    <t>q</t>
   </si>
   <si>
     <t>q@q</t>
   </si>
   <si>
-    <t>eie</t>
+    <t>Brother</t>
+  </si>
+  <si>
+    <t>mecheng</t>
+  </si>
+  <si>
+    <t>w</t>
   </si>
   <si>
     <t>w@w</t>
   </si>
   <si>
-    <t>Medicine</t>
+    <t>Sister</t>
+  </si>
+  <si>
+    <t>medicine</t>
+  </si>
+  <si>
+    <t>e</t>
   </si>
   <si>
     <t>e@e</t>
   </si>
   <si>
-    <t>Physics</t>
-  </si>
-  <si>
-    <t>r@r</t>
-  </si>
-  <si>
-    <t>Business</t>
-  </si>
-  <si>
-    <t>Econimics </t>
+    <t>maths</t>
+  </si>
+  <si>
+    <t>r</t>
+  </si>
+  <si>
+    <t>r@R</t>
+  </si>
+  <si>
+    <t>chemistry</t>
+  </si>
+  <si>
+    <t>t</t>
   </si>
   <si>
     <t>t@t</t>
   </si>
   <si>
-    <t>No</t>
+    <t>y</t>
   </si>
   <si>
     <t>y@y</t>
   </si>
   <si>
+    <t>u</t>
+  </si>
+  <si>
     <t>u@u</t>
   </si>
   <si>
-    <t>Chemistry</t>
+    <t>i</t>
   </si>
   <si>
     <t>i@i</t>
-  </si>
-  <si>
-    <t>Maths</t>
-  </si>
-  <si>
-    <t>o@O</t>
-  </si>
-  <si>
-    <t>Finance </t>
-  </si>
-  <si>
-    <t>email2</t>
   </si>
 </sst>
 </file>
@@ -178,16 +169,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
+  <dxfs count="10">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -232,22 +214,19 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:M11" totalsRowShown="0">
-  <autoFilter ref="A1:M11" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Start time" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Completion time" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Email" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Name" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Last modified time" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="email2" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Faculty " dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Engineerings" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Medicines" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="NatSci" dataDxfId="2"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Business " dataDxfId="1"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Okay with someone in Faculty but not desired course? " dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:J9" totalsRowShown="0">
+  <autoFilter ref="A1:J9" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="10">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Start time" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Completion time" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Email" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Name" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Last modified time" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Name2" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Email2" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Gender" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Course applying for" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -550,13 +529,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="13" width="20" bestFit="1" customWidth="1"/>
+    <col min="1" max="10" width="20" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -576,93 +555,84 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" s="1">
-        <v>46263.720104166663</v>
+        <v>46263.81726851852</v>
       </c>
       <c r="C2" s="1">
-        <v>46263.720381944448</v>
+        <v>46263.817442129628</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" t="s">
         <v>13</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>14</v>
       </c>
-      <c r="I2" t="s">
-        <v>15</v>
-      </c>
-      <c r="M2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" s="1">
-        <v>46263.724733796298</v>
+        <v>46263.817453703705</v>
       </c>
       <c r="C3" s="1">
-        <v>46263.725069444445</v>
+        <v>46263.81753472222</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" t="s">
         <v>17</v>
       </c>
-      <c r="H3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>18</v>
       </c>
-      <c r="M3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" s="1">
-        <v>46263.725081018521</v>
+        <v>46263.817557870374</v>
       </c>
       <c r="C4" s="1">
-        <v>46263.725208333337</v>
+        <v>46263.817627314813</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" t="s">
@@ -671,200 +641,146 @@
       <c r="H4" t="s">
         <v>20</v>
       </c>
+      <c r="I4" t="s">
+        <v>13</v>
+      </c>
       <c r="J4" t="s">
-        <v>20</v>
-      </c>
-      <c r="M4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" s="1">
-        <v>46263.725219907406</v>
+        <v>46263.81763888889</v>
       </c>
       <c r="C5" s="1">
-        <v>46263.725324074076</v>
+        <v>46263.817708333336</v>
       </c>
       <c r="D5" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H5" t="s">
-        <v>9</v>
-      </c>
-      <c r="K5" t="s">
-        <v>22</v>
-      </c>
-      <c r="M5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" s="1">
-        <v>46263.725347222222</v>
+        <v>46263.817731481482</v>
       </c>
       <c r="C6" s="1">
-        <v>46263.725497685184</v>
+        <v>46263.817870370367</v>
       </c>
       <c r="D6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H6" t="s">
-        <v>24</v>
-      </c>
-      <c r="L6" t="s">
-        <v>25</v>
-      </c>
-      <c r="M6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+        <v>26</v>
+      </c>
+      <c r="I6" t="s">
+        <v>17</v>
+      </c>
+      <c r="J6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" s="1">
-        <v>46263.72550925926</v>
+        <v>46263.817893518521</v>
       </c>
       <c r="C7" s="1">
-        <v>46263.725601851853</v>
+        <v>46263.817986111113</v>
       </c>
       <c r="D7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H7" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="I7" t="s">
-        <v>15</v>
-      </c>
-      <c r="M7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+      <c r="J7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" s="1">
-        <v>46263.725624999999</v>
+        <v>46263.818009259259</v>
       </c>
       <c r="C8" s="1">
-        <v>46263.725694444445</v>
+        <v>46263.818090277775</v>
       </c>
       <c r="D8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H8" t="s">
-        <v>20</v>
+        <v>30</v>
+      </c>
+      <c r="I8" t="s">
+        <v>17</v>
       </c>
       <c r="J8" t="s">
-        <v>20</v>
-      </c>
-      <c r="M8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" s="1">
-        <v>46263.725717592592</v>
+        <v>46263.818101851852</v>
       </c>
       <c r="C9" s="1">
-        <v>46263.725821759261</v>
+        <v>46263.818206018521</v>
       </c>
       <c r="D9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H9" t="s">
-        <v>9</v>
-      </c>
-      <c r="K9" t="s">
-        <v>30</v>
-      </c>
-      <c r="M9" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" s="1">
-        <v>46263.72583333333</v>
-      </c>
-      <c r="C10" s="1">
-        <v>46263.725914351853</v>
-      </c>
-      <c r="D10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="1"/>
-      <c r="G10" t="s">
-        <v>31</v>
-      </c>
-      <c r="H10" t="s">
-        <v>9</v>
-      </c>
-      <c r="K10" t="s">
         <v>32</v>
       </c>
-      <c r="M10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" s="1">
-        <v>46263.725925925923</v>
-      </c>
-      <c r="C11" s="1">
-        <v>46263.726041666669</v>
-      </c>
-      <c r="D11" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="1"/>
-      <c r="G11" t="s">
-        <v>33</v>
-      </c>
-      <c r="H11" t="s">
+      <c r="I9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J9" t="s">
         <v>24</v>
-      </c>
-      <c r="L11" t="s">
-        <v>34</v>
-      </c>
-      <c r="M11" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>